<commit_message>
Update logs_labs1.xlsx with latest edits
</commit_message>
<xml_diff>
--- a/logs_labs1.xlsx
+++ b/logs_labs1.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\khadjia\Desktop\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E2BFCFBB-5815-462B-BB09-C6F9B5704A13}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CEE5BDC4-F47A-4380-BE79-FF75B60B9B17}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{E1B0EFE5-83BB-46EC-A35E-DF12770E8C81}"/>
   </bookViews>
@@ -58,9 +58,6 @@
     <t>Impossible de créer une politique de mise à l’échelle pour un groupe Auto Scaling EC2.                                                   Le service indique que le rôle IAM lié au service n’est pas encore disponible.</t>
   </si>
   <si>
-    <t>Erreur lors de la création de la politique de scaling :                                                     « EC2 Auto Scaling n’a pas l’autorisation requise ».                                                             Le groupe Auto Scaling est créé correctement, mais la politique de scaling échoue.</t>
-  </si>
-  <si>
     <t>Le rôle IAM lié au service Auto Scaling (Service‑Linked Role) n’est pas encore entièrement propagé au moment de la création de la politique.
 Un délai est nécessaire pour que le rôle soit utilisable par les services AWS.</t>
   </si>
@@ -80,6 +77,9 @@
   <si>
     <t>Problème temporaire fréquent lié à la propagation des rôles IAM.
 Il se résout généralement sans intervention technique complexe.</t>
+  </si>
+  <si>
+    <t>Erreur lors de la création de la politique de scaling :                                                                « EC2 Auto Scaling n’a pas l’autorisation requise ».                                                             Le groupe Auto Scaling est créé correctement, mais la politique de scaling échoue.</t>
   </si>
 </sst>
 </file>
@@ -1000,19 +1000,19 @@
         <v>10</v>
       </c>
       <c r="D2" s="5" t="s">
+        <v>15</v>
+      </c>
+      <c r="E2" s="5" t="s">
         <v>11</v>
       </c>
-      <c r="E2" s="5" t="s">
+      <c r="F2" s="5" t="s">
         <v>12</v>
       </c>
-      <c r="F2" s="5" t="s">
+      <c r="G2" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="G2" s="5" t="s">
+      <c r="H2" s="5" t="s">
         <v>14</v>
-      </c>
-      <c r="H2" s="5" t="s">
-        <v>15</v>
       </c>
     </row>
   </sheetData>

</xml_diff>